<commit_message>
adapt due r4 change
</commit_message>
<xml_diff>
--- a/011/ranks.xlsx
+++ b/011/ranks.xlsx
@@ -386,7 +386,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -407,11 +407,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -480,7 +475,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -498,10 +493,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2241,7 +2232,7 @@
       <c r="A66" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="4" t="s">
         <v>77</v>
       </c>
       <c r="C66" s="2" t="n">
@@ -2351,7 +2342,7 @@
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C71" s="2" t="n">
@@ -2428,7 +2419,7 @@
         <f aca="false">VLOOKUP(B74,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E74" s="6" t="s">
+      <c r="E74" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F74" s="1" t="str">
@@ -2450,7 +2441,7 @@
         <f aca="false">VLOOKUP(B75,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E75" s="6" t="s">
+      <c r="E75" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F75" s="1" t="str">
@@ -2472,7 +2463,7 @@
         <f aca="false">VLOOKUP(B76,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E76" s="6" t="s">
+      <c r="E76" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F76" s="1" t="str">
@@ -2494,7 +2485,7 @@
         <f aca="false">VLOOKUP(B77,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E77" s="6" t="s">
+      <c r="E77" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F77" s="1" t="str">
@@ -2539,7 +2530,7 @@
         <f aca="false">VLOOKUP(B79,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E79" s="6" t="s">
+      <c r="E79" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F79" s="1" t="str">
@@ -2583,7 +2574,7 @@
         <f aca="false">VLOOKUP(B81,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E81" s="6" t="s">
+      <c r="E81" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F81" s="1" t="str">
@@ -2605,7 +2596,7 @@
         <f aca="false">VLOOKUP(B82,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="E82" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F82" s="1" t="str">
@@ -2627,7 +2618,7 @@
         <f aca="false">VLOOKUP(B83,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E83" s="6" t="s">
+      <c r="E83" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F83" s="1" t="str">
@@ -2650,7 +2641,7 @@
         <f aca="false">VLOOKUP(B84,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E84" s="6" t="s">
+      <c r="E84" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F84" s="1" t="str">
@@ -2672,7 +2663,7 @@
         <f aca="false">VLOOKUP(B85,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E85" s="6" t="s">
+      <c r="E85" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F85" s="1" t="str">
@@ -2695,7 +2686,7 @@
         <f aca="false">VLOOKUP(B86,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E86" s="6" t="s">
+      <c r="E86" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F86" s="1" t="str">
@@ -2717,7 +2708,7 @@
         <f aca="false">VLOOKUP(B87,TS!$B$2:$D$99,2,0)</f>
         <v>R1</v>
       </c>
-      <c r="E87" s="6" t="s">
+      <c r="E87" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F87" s="1" t="str">
@@ -2739,7 +2730,7 @@
         <f aca="false">VLOOKUP(B88,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E88" s="6" t="s">
+      <c r="E88" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F88" s="1" t="str">
@@ -2761,7 +2752,7 @@
         <f aca="false">VLOOKUP(B89,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E89" s="7" t="s">
+      <c r="E89" s="6" t="s">
         <v>101</v>
       </c>
       <c r="F89" s="1" t="str">
@@ -2783,7 +2774,7 @@
         <f aca="false">VLOOKUP(B90,TS!$B$2:$D$99,2,0)</f>
         <v>R2</v>
       </c>
-      <c r="E90" s="7" t="s">
+      <c r="E90" s="6" t="s">
         <v>101</v>
       </c>
       <c r="F90" s="1" t="str">
@@ -2894,7 +2885,7 @@
         <f aca="false">VLOOKUP(B95,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E95" s="7" t="s">
+      <c r="E95" s="6" t="s">
         <v>101</v>
       </c>
       <c r="F95" s="1" t="str">
@@ -2961,7 +2952,7 @@
         <f aca="false">VLOOKUP(B98,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E98" s="7" t="s">
+      <c r="E98" s="6" t="s">
         <v>101</v>
       </c>
       <c r="F98" s="1" t="str">
@@ -2983,7 +2974,7 @@
         <f aca="false">VLOOKUP(B99,TS!$B$2:$D$99,2,0)</f>
         <v>R3</v>
       </c>
-      <c r="E99" s="7" t="s">
+      <c r="E99" s="6" t="s">
         <v>101</v>
       </c>
       <c r="F99" s="1" t="str">
@@ -3644,7 +3635,7 @@
       <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="4" t="s">
         <v>94</v>
       </c>
       <c r="C45" s="1" t="s">
@@ -3854,7 +3845,7 @@
       <c r="A60" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C60" s="1" t="s">

</xml_diff>